<commit_message>
v7.3.86-4: Fehlzeiten-Bug gefixt, Header-Navigation entfernt, Umlaute korrigiert
</commit_message>
<xml_diff>
--- a/Vorlagen/AP IMPORT Projektplan_2025-2027.xlsx
+++ b/Vorlagen/AP IMPORT Projektplan_2025-2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdbs/Documents/Dev/projektzeiterfassung20/Vorlagen/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdbs/Documents/Dev/PZE/Vorlagen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37C93F95-56D9-F646-8CE5-05BB6C869044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D795446E-8403-5B45-B425-130FB1D9E579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15900" yWindow="-28180" windowWidth="51200" windowHeight="28180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15120" yWindow="-21000" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projektplan" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Projektplan!$A$1:$D$46</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="85">
   <si>
     <t>Nr.</t>
   </si>
@@ -275,6 +275,32 @@
   </si>
   <si>
     <t>Summe</t>
+  </si>
+  <si>
+    <t>AP-Nr.</t>
+  </si>
+  <si>
+    <t>Kurzbeschreibung</t>
+  </si>
+  <si>
+    <t>MA-Nr 1
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 2
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 3
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 4
+PM</t>
+  </si>
+  <si>
+    <t>AP
+Summe PM</t>
   </si>
 </sst>
 </file>
@@ -342,28 +368,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,6 +477,58 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>415958</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Grafik 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{716EE0CF-55F4-E219-38F2-C0A541385B49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="26149300" y="2654300"/>
+          <a:ext cx="7772400" cy="1381158"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -629,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:AA48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="74" customWidth="1"/>
@@ -637,10 +718,12 @@
     <col min="11" max="11" width="6.5" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="52.1640625" style="5" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="13.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="14.1640625" style="5"/>
+    <col min="15" max="19" width="14.1640625" style="5"/>
+    <col min="20" max="20" width="30" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="14.1640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" ht="95" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" s="2" customFormat="1" ht="95" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -671,8 +754,35 @@
       <c r="P1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+      <c r="S1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="57" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -697,8 +807,36 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:16" ht="38" x14ac:dyDescent="0.2">
+      <c r="S2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="T2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="W2" s="3">
+        <v>1</v>
+      </c>
+      <c r="X2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA2" s="3">
+        <f>SUM(W2:Z2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="38" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -732,7 +870,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="19" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -764,7 +902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="57" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="57" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>29</v>
       </c>
@@ -798,7 +936,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="19" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
@@ -830,7 +968,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="38" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" ht="38" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>37</v>
       </c>
@@ -864,7 +1002,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" ht="19" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
@@ -896,7 +1034,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" ht="19" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>47</v>
       </c>
@@ -928,7 +1066,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="38" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" ht="38" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>51</v>
       </c>
@@ -954,7 +1092,7 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
     </row>
-    <row r="11" spans="1:16" ht="38" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" ht="38" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>55</v>
       </c>
@@ -980,7 +1118,7 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
     </row>
-    <row r="12" spans="1:16" ht="76" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" ht="76" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>59</v>
       </c>
@@ -1006,7 +1144,7 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
     </row>
-    <row r="13" spans="1:16" ht="76" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" ht="76" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>65</v>
       </c>
@@ -1032,7 +1170,7 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
     </row>
-    <row r="14" spans="1:16" ht="76" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" ht="76" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>69</v>
       </c>
@@ -1066,7 +1204,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" ht="19" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>73</v>
       </c>
@@ -1098,7 +1236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="9"/>
@@ -1891,5 +2029,6 @@
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v7.3.87: Arbeitsplan Excel Import Feature
NEUE FEATURES:
- Projekt-Team Management: MA aus Firma auswählen + lfd. Nr. vergeben
- Excel-Vorlage Download: Projektspezifisch mit MA-Namen und Nummern
- Excel-Import: Arbeitspakete aus Excel importieren mit Vorschau

NEUE KOMPONENTEN:
- ProjectTeamManager.tsx: Team-Tab im Projekt (ersetzt alte Team-Tabelle)
- ArbeitsplanImport.tsx: Download/Upload Buttons + Import-Dialog

AKTUALISIERTE KOMPONENTEN:
- ProjectDetailPage.tsx: Integriert Team-Manager und Import-Buttons

NEUE API ROUTES:
- /api/v7/arbeitsplan-vorlage: Generiert projektspezifische Excel-Vorlage
- /api/v7/arbeitsplan-import: Parst Excel und importiert APs

ABHÄNGIGKEITEN:
- exceljs (npm install exceljs)

WICHTIG: Nach Deployment DB-Migration ausführen!
</commit_message>
<xml_diff>
--- a/Vorlagen/AP IMPORT Projektplan_2025-2027.xlsx
+++ b/Vorlagen/AP IMPORT Projektplan_2025-2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdbs/Documents/Dev/PZE/Vorlagen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D795446E-8403-5B45-B425-130FB1D9E579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942745BC-85B3-744C-9E7C-2655FD8A6905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="-21000" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19560" yWindow="-25300" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projektplan" sheetId="1" r:id="rId1"/>
@@ -283,24 +283,28 @@
     <t>Kurzbeschreibung</t>
   </si>
   <si>
-    <t>MA-Nr 1
-PM</t>
-  </si>
-  <si>
-    <t>MA-Nr 2
-PM</t>
-  </si>
-  <si>
-    <t>MA-Nr 3
-PM</t>
-  </si>
-  <si>
-    <t>MA-Nr 4
-PM</t>
-  </si>
-  <si>
     <t>AP
 Summe PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 1
+V.Name
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 2
+V.Name
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 3
+V.Name
+PM</t>
+  </si>
+  <si>
+    <t>MA-Nr 4
+V.Name
+PM</t>
   </si>
 </sst>
 </file>
@@ -481,53 +485,64 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>415958</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Grafik 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{716EE0CF-55F4-E219-38F2-C0A541385B49}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="26149300" y="2654300"/>
-          <a:ext cx="7772400" cy="1381158"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>18</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>12700</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>27</xdr:col>
+          <xdr:colOff>12700</xdr:colOff>
+          <xdr:row>9</xdr:row>
+          <xdr:rowOff>25400</xdr:rowOff>
+        </xdr:to>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="2" name="Grafik 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E232B7A0-389B-9177-DBFD-71B551E8F572}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="$S$1:$AA$2" spid="_x0000_s1029"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="26149300" y="2667000"/>
+              <a:ext cx="10934700" cy="1943100"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -709,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
@@ -767,19 +782,19 @@
         <v>3</v>
       </c>
       <c r="W1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="57" x14ac:dyDescent="0.2">
@@ -2030,5 +2045,6 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>